<commit_message>
Actualización automática: 2026-04-22 15:45:38
</commit_message>
<xml_diff>
--- a/cis_auditoria/_audit_reports/Audit_EC2-WEST2-BASTION-CORBETA_35.86.158.63.xlsx
+++ b/cis_auditoria/_audit_reports/Audit_EC2-WEST2-BASTION-CORBETA_35.86.158.63.xlsx
@@ -36,7 +36,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -58,11 +58,6 @@
         <fgColor rgb="00E7E6E6"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -76,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -91,9 +86,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -561,7 +553,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C4" s="3" t="n"/>
       <c r="D4" s="3" t="n"/>
@@ -584,7 +576,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5" s="3" t="n"/>
       <c r="D5" s="3" t="n"/>
@@ -8749,14 +8741,14 @@
           <t>Valida que SSH tenga configurado un banner distinto de none; si existe → cumple, si no → no cumple.</t>
         </is>
       </c>
-      <c r="I136" s="6" t="inlineStr">
-        <is>
-          <t>No cumple</t>
+      <c r="I136" s="4" t="inlineStr">
+        <is>
+          <t>Cumple</t>
         </is>
       </c>
       <c r="J136" s="3" t="inlineStr">
         <is>
-          <t>banner /etc/issue.net</t>
+          <t>Banner /etc/issue.net</t>
         </is>
       </c>
       <c r="K136" s="3" t="inlineStr"/>
@@ -8765,7 +8757,7 @@
       </c>
       <c r="M136" s="3" t="inlineStr">
         <is>
-          <t>banner /etc/issue.net</t>
+          <t>Banner /etc/issue.net</t>
         </is>
       </c>
       <c r="N136" s="3" t="inlineStr"/>

</xml_diff>